<commit_message>
correcoes da terceira revisao pedro
</commit_message>
<xml_diff>
--- a/avaliacao/Pedro/ouro_Pedro.xlsx
+++ b/avaliacao/Pedro/ouro_Pedro.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30430"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\extrator_fragmentos_leis\avaliacao\Pedro\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{28200485-0D83-4467-9F91-3977580A391A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CAEA9301-31FA-4229-9951-9876AABD2D1E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9910" uniqueCount="2008">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9910" uniqueCount="2007">
   <si>
     <t>campo</t>
   </si>
@@ -6034,9 +6034,6 @@
     <t>revisada</t>
   </si>
   <si>
-    <t>Precisei adicionar o Fecho</t>
-  </si>
-  <si>
     <t>Havia o simbolo ( --&gt;) no final do FECHO. O simbolo foi removido</t>
   </si>
   <si>
@@ -6049,7 +6046,7 @@
     <t>corrigir</t>
   </si>
   <si>
-    <t>Precisei adicionar a ementa</t>
+    <t>Precisei adicionar o Fecho no Json</t>
   </si>
 </sst>
 </file>
@@ -6576,7 +6573,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:11" s="18" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:11" s="18" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A2" s="12" t="s">
         <v>20</v>
       </c>
@@ -6686,7 +6683,7 @@
         <v>1995</v>
       </c>
     </row>
-    <row r="6" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A6" s="16" t="s">
         <v>24</v>
       </c>
@@ -6853,7 +6850,7 @@
       </c>
       <c r="K11" s="6"/>
     </row>
-    <row r="12" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A12" s="16" t="s">
         <v>30</v>
       </c>
@@ -6873,7 +6870,7 @@
         <v>395</v>
       </c>
       <c r="G12" s="13" t="s">
-        <v>2002</v>
+        <v>2006</v>
       </c>
       <c r="H12" s="13" t="s">
         <v>2000</v>
@@ -7174,7 +7171,7 @@
         <v>395</v>
       </c>
       <c r="G23" s="13" t="s">
-        <v>2003</v>
+        <v>2002</v>
       </c>
       <c r="H23" s="13" t="s">
         <v>1994</v>
@@ -7909,7 +7906,7 @@
         <v>395</v>
       </c>
       <c r="G50" s="13" t="s">
-        <v>2003</v>
+        <v>2002</v>
       </c>
       <c r="H50" s="13" t="s">
         <v>1994</v>
@@ -8458,7 +8455,7 @@
         <v>1995</v>
       </c>
     </row>
-    <row r="71" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A71" s="2" t="s">
         <v>124</v>
       </c>
@@ -8485,7 +8482,7 @@
         <v>1995</v>
       </c>
     </row>
-    <row r="72" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A72" s="2" t="s">
         <v>129</v>
       </c>
@@ -8512,7 +8509,7 @@
         <v>1995</v>
       </c>
     </row>
-    <row r="73" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A73" s="2" t="s">
         <v>130</v>
       </c>
@@ -8539,7 +8536,7 @@
         <v>1995</v>
       </c>
     </row>
-    <row r="74" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A74" s="2" t="s">
         <v>131</v>
       </c>
@@ -8566,7 +8563,7 @@
         <v>1995</v>
       </c>
     </row>
-    <row r="75" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A75" s="2" t="s">
         <v>132</v>
       </c>
@@ -8593,7 +8590,7 @@
         <v>1995</v>
       </c>
     </row>
-    <row r="76" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A76" s="2" t="s">
         <v>134</v>
       </c>
@@ -8620,7 +8617,7 @@
         <v>1995</v>
       </c>
     </row>
-    <row r="77" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A77" s="2" t="s">
         <v>135</v>
       </c>
@@ -8647,7 +8644,7 @@
         <v>1995</v>
       </c>
     </row>
-    <row r="78" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A78" s="2" t="s">
         <v>138</v>
       </c>
@@ -8674,7 +8671,7 @@
         <v>1995</v>
       </c>
     </row>
-    <row r="79" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A79" s="2" t="s">
         <v>141</v>
       </c>
@@ -8701,7 +8698,7 @@
         <v>1995</v>
       </c>
     </row>
-    <row r="80" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A80" s="2" t="s">
         <v>142</v>
       </c>
@@ -8728,7 +8725,7 @@
         <v>1995</v>
       </c>
     </row>
-    <row r="81" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A81" s="2" t="s">
         <v>143</v>
       </c>
@@ -8755,7 +8752,7 @@
         <v>1995</v>
       </c>
     </row>
-    <row r="82" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A82" s="2" t="s">
         <v>144</v>
       </c>
@@ -8802,7 +8799,7 @@
         <v>395</v>
       </c>
       <c r="G83" s="13" t="s">
-        <v>2002</v>
+        <v>2006</v>
       </c>
       <c r="H83" s="13" t="s">
         <v>2000</v>
@@ -8811,7 +8808,7 @@
         <v>1995</v>
       </c>
     </row>
-    <row r="84" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A84" s="2" t="s">
         <v>118</v>
       </c>
@@ -8838,7 +8835,7 @@
         <v>1995</v>
       </c>
     </row>
-    <row r="85" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A85" t="s">
         <v>120</v>
       </c>
@@ -8865,7 +8862,7 @@
         <v>1995</v>
       </c>
     </row>
-    <row r="86" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A86" t="s">
         <v>121</v>
       </c>
@@ -8892,7 +8889,7 @@
         <v>1995</v>
       </c>
     </row>
-    <row r="87" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A87" t="s">
         <v>122</v>
       </c>
@@ -8919,7 +8916,7 @@
         <v>1995</v>
       </c>
     </row>
-    <row r="88" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A88" t="s">
         <v>123</v>
       </c>
@@ -8946,7 +8943,7 @@
         <v>1995</v>
       </c>
     </row>
-    <row r="89" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A89" t="s">
         <v>125</v>
       </c>
@@ -8974,7 +8971,7 @@
       </c>
     </row>
     <row r="90" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A90" t="s">
+      <c r="A90" s="13" t="s">
         <v>126</v>
       </c>
       <c r="B90" s="13">
@@ -8992,8 +8989,8 @@
       <c r="F90" s="13" t="s">
         <v>395</v>
       </c>
-      <c r="G90" s="13" t="s">
-        <v>2007</v>
+      <c r="G90" s="16" t="s">
+        <v>1999</v>
       </c>
       <c r="H90" s="13" t="s">
         <v>2000</v>
@@ -9003,7 +9000,7 @@
       </c>
     </row>
     <row r="91" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A91" t="s">
+      <c r="A91" s="13" t="s">
         <v>127</v>
       </c>
       <c r="B91" s="13">
@@ -9022,7 +9019,7 @@
         <v>395</v>
       </c>
       <c r="G91" s="13" t="s">
-        <v>2007</v>
+        <v>1999</v>
       </c>
       <c r="H91" s="13" t="s">
         <v>2000</v>
@@ -9032,7 +9029,7 @@
       </c>
     </row>
     <row r="92" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A92" t="s">
+      <c r="A92" s="13" t="s">
         <v>128</v>
       </c>
       <c r="B92" s="13">
@@ -9051,7 +9048,7 @@
         <v>395</v>
       </c>
       <c r="G92" s="13" t="s">
-        <v>2007</v>
+        <v>1999</v>
       </c>
       <c r="H92" s="13" t="s">
         <v>2000</v>
@@ -9060,7 +9057,7 @@
         <v>1995</v>
       </c>
     </row>
-    <row r="93" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A93" t="s">
         <v>133</v>
       </c>
@@ -9087,7 +9084,7 @@
         <v>1995</v>
       </c>
     </row>
-    <row r="94" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A94" t="s">
         <v>136</v>
       </c>
@@ -9114,7 +9111,7 @@
         <v>1995</v>
       </c>
     </row>
-    <row r="95" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="95" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A95" t="s">
         <v>137</v>
       </c>
@@ -9141,7 +9138,7 @@
         <v>1995</v>
       </c>
     </row>
-    <row r="96" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A96" t="s">
         <v>139</v>
       </c>
@@ -9168,7 +9165,7 @@
         <v>1995</v>
       </c>
     </row>
-    <row r="97" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="97" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A97" t="s">
         <v>140</v>
       </c>
@@ -9195,7 +9192,7 @@
         <v>1995</v>
       </c>
     </row>
-    <row r="98" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="98" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A98" t="s">
         <v>108</v>
       </c>
@@ -9219,7 +9216,7 @@
         <v>401</v>
       </c>
     </row>
-    <row r="99" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="99" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A99" t="s">
         <v>110</v>
       </c>
@@ -9243,7 +9240,7 @@
         <v>401</v>
       </c>
     </row>
-    <row r="100" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="100" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A100" t="s">
         <v>111</v>
       </c>
@@ -9267,7 +9264,7 @@
         <v>401</v>
       </c>
     </row>
-    <row r="101" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="101" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A101" t="s">
         <v>113</v>
       </c>
@@ -9291,7 +9288,7 @@
         <v>401</v>
       </c>
     </row>
-    <row r="102" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="102" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A102" t="s">
         <v>114</v>
       </c>
@@ -9315,7 +9312,7 @@
         <v>401</v>
       </c>
     </row>
-    <row r="103" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="103" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A103" t="s">
         <v>116</v>
       </c>
@@ -9339,7 +9336,7 @@
         <v>401</v>
       </c>
     </row>
-    <row r="104" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="104" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A104" t="s">
         <v>117</v>
       </c>
@@ -9363,7 +9360,7 @@
         <v>401</v>
       </c>
     </row>
-    <row r="105" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="105" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A105" t="s">
         <v>119</v>
       </c>
@@ -9387,7 +9384,7 @@
         <v>401</v>
       </c>
     </row>
-    <row r="106" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="106" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A106" t="s">
         <v>109</v>
       </c>
@@ -9411,7 +9408,7 @@
         <v>401</v>
       </c>
     </row>
-    <row r="107" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="107" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A107" t="s">
         <v>112</v>
       </c>
@@ -9435,7 +9432,7 @@
         <v>401</v>
       </c>
     </row>
-    <row r="108" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="108" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A108" t="s">
         <v>89</v>
       </c>
@@ -9459,7 +9456,7 @@
         <v>401</v>
       </c>
     </row>
-    <row r="109" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="109" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A109" t="s">
         <v>93</v>
       </c>
@@ -9483,7 +9480,7 @@
         <v>401</v>
       </c>
     </row>
-    <row r="110" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="110" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A110" t="s">
         <v>97</v>
       </c>
@@ -9507,7 +9504,7 @@
         <v>401</v>
       </c>
     </row>
-    <row r="111" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="111" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A111" t="s">
         <v>106</v>
       </c>
@@ -9531,7 +9528,7 @@
         <v>401</v>
       </c>
     </row>
-    <row r="112" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="112" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A112" t="s">
         <v>91</v>
       </c>
@@ -9555,7 +9552,7 @@
         <v>401</v>
       </c>
     </row>
-    <row r="113" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="113" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A113" t="s">
         <v>99</v>
       </c>
@@ -9579,7 +9576,7 @@
         <v>401</v>
       </c>
     </row>
-    <row r="114" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="114" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A114" t="s">
         <v>90</v>
       </c>
@@ -9603,7 +9600,7 @@
         <v>401</v>
       </c>
     </row>
-    <row r="115" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="115" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A115" t="s">
         <v>105</v>
       </c>
@@ -9627,7 +9624,7 @@
         <v>401</v>
       </c>
     </row>
-    <row r="116" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="116" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A116" t="s">
         <v>107</v>
       </c>
@@ -9651,7 +9648,7 @@
         <v>401</v>
       </c>
     </row>
-    <row r="117" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="117" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A117" t="s">
         <v>103</v>
       </c>
@@ -9675,7 +9672,7 @@
         <v>401</v>
       </c>
     </row>
-    <row r="118" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="118" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A118" t="s">
         <v>102</v>
       </c>
@@ -9699,7 +9696,7 @@
         <v>401</v>
       </c>
     </row>
-    <row r="119" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="119" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A119" t="s">
         <v>95</v>
       </c>
@@ -9723,7 +9720,7 @@
         <v>401</v>
       </c>
     </row>
-    <row r="120" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="120" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A120" t="s">
         <v>100</v>
       </c>
@@ -9747,7 +9744,7 @@
         <v>401</v>
       </c>
     </row>
-    <row r="121" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="121" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A121" t="s">
         <v>92</v>
       </c>
@@ -9771,7 +9768,7 @@
         <v>401</v>
       </c>
     </row>
-    <row r="122" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="122" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A122" t="s">
         <v>98</v>
       </c>
@@ -9795,7 +9792,7 @@
         <v>401</v>
       </c>
     </row>
-    <row r="123" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="123" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A123" t="s">
         <v>104</v>
       </c>
@@ -9819,7 +9816,7 @@
         <v>401</v>
       </c>
     </row>
-    <row r="124" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="124" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A124" t="s">
         <v>101</v>
       </c>
@@ -9843,7 +9840,7 @@
         <v>401</v>
       </c>
     </row>
-    <row r="125" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="125" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A125" t="s">
         <v>94</v>
       </c>
@@ -9867,7 +9864,7 @@
         <v>401</v>
       </c>
     </row>
-    <row r="126" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="126" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A126" t="s">
         <v>96</v>
       </c>
@@ -9896,9 +9893,11 @@
     </row>
   </sheetData>
   <autoFilter ref="A1:I126" xr:uid="{00000000-0001-0000-0100-000000000000}">
-    <filterColumn colId="8">
+    <filterColumn colId="6">
       <filters>
-        <filter val="pendente de revisão humana"/>
+        <filter val="Precisei adicionar a ementa"/>
+        <filter val="Precisei adicionar o Fecho"/>
+        <filter val="Precisei incluir a ementa no Json"/>
       </filters>
     </filterColumn>
     <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A71:I126">
@@ -21040,7 +21039,7 @@
         <v>39</v>
       </c>
       <c r="C357" s="15" t="s">
-        <v>2004</v>
+        <v>2003</v>
       </c>
       <c r="D357" s="2" t="s">
         <v>411</v>
@@ -21056,7 +21055,7 @@
         <v>1298</v>
       </c>
       <c r="I357" s="15" t="s">
-        <v>2005</v>
+        <v>2004</v>
       </c>
       <c r="J357" s="2" t="s">
         <v>1992</v>
@@ -42703,7 +42702,7 @@
         <v>3</v>
       </c>
       <c r="C1128" s="13" t="s">
-        <v>2006</v>
+        <v>2005</v>
       </c>
       <c r="D1128" s="13" t="s">
         <v>411</v>

</xml_diff>